<commit_message>
feat(create): unify employee and vendor management with common modules and shared base
</commit_message>
<xml_diff>
--- a/swarajya-create/employee-management/test_data/Swarajya-Create-test-cases (6).xlsx
+++ b/swarajya-create/employee-management/test_data/Swarajya-Create-test-cases (6).xlsx
@@ -29003,12 +29003,12 @@
       </c>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>Application defect: Form failed to display mandatory Department validation error message upon submission</t>
+          <t>Validation successful: Form rejected invalid input and prevented submission.</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
@@ -29395,12 +29395,12 @@
       </c>
       <c r="J18" s="10" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>Validation successful: Form rejected invalid input and prevented submission.</t>
+          <t>ModuleNotFoundError: No module named 'pages'</t>
         </is>
       </c>
       <c r="L18" s="7" t="inlineStr">

</xml_diff>